<commit_message>
feat: add intelligence engine and debugger workflow understanding
</commit_message>
<xml_diff>
--- a/uploads/test.xlsx
+++ b/uploads/test.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haozh\workspace\ai-bid-system\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haozh\workspace\ai-construction-system\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CB66EF5-1AE9-4D9B-A8DC-4E0093FBB9AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35FE5992-611B-4C45-BFB2-E9325651CA5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6600" yWindow="13510" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8290" yWindow="5510" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>项目名称</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -40,6 +40,10 @@
   </si>
   <si>
     <t>混凝土</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>钢筋</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -365,7 +369,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -388,6 +392,17 @@
       </c>
       <c r="C2">
         <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>5000</v>
+      </c>
+      <c r="C3">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(parser): add continuation row semantic detection
</commit_message>
<xml_diff>
--- a/uploads/test.xlsx
+++ b/uploads/test.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haozh\workspace\ai-construction-system\uploads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\haozh\workspace\ai-bid-system\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35FE5992-611B-4C45-BFB2-E9325651CA5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CB66EF5-1AE9-4D9B-A8DC-4E0093FBB9AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8290" yWindow="5510" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6600" yWindow="13510" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>项目名称</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -40,10 +40,6 @@
   </si>
   <si>
     <t>混凝土</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>钢筋</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -369,7 +365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -392,17 +388,6 @@
       </c>
       <c r="C2">
         <v>100</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3">
-        <v>5000</v>
-      </c>
-      <c r="C3">
-        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>